<commit_message>
Best Lifter: Pluralize title + No Plaque template
</commit_message>
<xml_diff>
--- a/local/templates/competitionBook/BestLifter.xlsx
+++ b/local/templates/competitionBook/BestLifter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/Misc/usaw-owlcms/local/templates/competitionBook/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Library/Application Support/owlcms/64.0.2+quick-start/local/templates/competitionBook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF57EB8-AB56-FA40-B750-D733BCBB1D82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDEA9481-7F18-7949-880B-C37C5C4F7DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18040" yWindow="1240" windowWidth="39500" windowHeight="25100" xr2:uid="{C695CBD2-3DAD-B341-8FFD-602D797EB14F}"/>
+    <workbookView xWindow="1540" yWindow="660" windowWidth="33020" windowHeight="21680" xr2:uid="{C695CBD2-3DAD-B341-8FFD-602D797EB14F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -371,9 +371,6 @@
     <t>${athlete.total == 0 ? "DNF" : athlete.bestLifterScore}</t>
   </si>
   <si>
-    <t>${mBest.0.ageGroup.championshipName} - Best Lifter</t>
-  </si>
-  <si>
     <t>Women</t>
   </si>
   <si>
@@ -387,6 +384,9 @@
   </si>
   <si>
     <t>${athlete.team}</t>
+  </si>
+  <si>
+    <t>${mBest.0.ageGroup.championshipName} - Best Lifters</t>
   </si>
 </sst>
 </file>
@@ -949,7 +949,7 @@
     </row>
     <row r="2" spans="1:16" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="16" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -987,7 +987,7 @@
     </row>
     <row r="4" spans="1:16" s="12" customFormat="1" ht="19" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
@@ -1059,7 +1059,7 @@
         <v>16</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>15</v>
@@ -1082,7 +1082,7 @@
     </row>
     <row r="10" spans="1:16" s="12" customFormat="1" ht="19" x14ac:dyDescent="0.2">
       <c r="A10" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
@@ -1143,7 +1143,7 @@
         <v>10</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -1154,7 +1154,7 @@
         <v>16</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>15</v>

</xml_diff>